<commit_message>
fix bugs, add BLT, BLTU
</commit_message>
<xml_diff>
--- a/Tomasulo3CPU/ISA/ISA64.xlsx
+++ b/Tomasulo3CPU/ISA/ISA64.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="RISCV64" sheetId="1" state="visible" r:id="rId3"/>
@@ -72,7 +72,25 @@
     <t xml:space="preserve">IMM[11]</t>
   </si>
   <si>
-    <t xml:space="preserve">U-TYPE: upper immediate instructions</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">U-TYPE: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">LUI / AUIPC</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">IMM[31:12]</t>
@@ -671,7 +689,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -693,6 +711,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -758,44 +782,48 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -991,564 +1019,564 @@
   <dimension ref="A1:AF29"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="1" style="0" width="7.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="1" style="1" width="7.33"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="n">
+      <c r="A1" s="1" t="n">
         <v>31</v>
       </c>
-      <c r="B1" s="0" t="n">
+      <c r="B1" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="C1" s="0" t="n">
+      <c r="C1" s="1" t="n">
         <v>29</v>
       </c>
-      <c r="D1" s="0" t="n">
+      <c r="D1" s="1" t="n">
         <v>28</v>
       </c>
-      <c r="E1" s="0" t="n">
+      <c r="E1" s="1" t="n">
         <v>27</v>
       </c>
-      <c r="F1" s="0" t="n">
+      <c r="F1" s="1" t="n">
         <v>26</v>
       </c>
-      <c r="G1" s="0" t="n">
+      <c r="G1" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="H1" s="0" t="n">
+      <c r="H1" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="I1" s="0" t="n">
+      <c r="I1" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="J1" s="0" t="n">
+      <c r="J1" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="K1" s="0" t="n">
+      <c r="K1" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="L1" s="0" t="n">
+      <c r="L1" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="M1" s="0" t="n">
+      <c r="M1" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="N1" s="0" t="n">
+      <c r="N1" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="O1" s="0" t="n">
+      <c r="O1" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="P1" s="0" t="n">
+      <c r="P1" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="Q1" s="0" t="n">
+      <c r="Q1" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="R1" s="0" t="n">
+      <c r="R1" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="S1" s="0" t="n">
+      <c r="S1" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="T1" s="0" t="n">
+      <c r="T1" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="U1" s="0" t="n">
+      <c r="U1" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="V1" s="0" t="n">
+      <c r="V1" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="W1" s="0" t="n">
+      <c r="W1" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="X1" s="0" t="n">
+      <c r="X1" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="Y1" s="0" t="n">
+      <c r="Y1" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="Z1" s="0" t="n">
+      <c r="Z1" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="AA1" s="0" t="n">
+      <c r="AA1" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="AB1" s="0" t="n">
+      <c r="AB1" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="AC1" s="0" t="n">
+      <c r="AC1" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="AD1" s="0" t="n">
+      <c r="AD1" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="AE1" s="0" t="n">
+      <c r="AE1" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AF1" s="0" t="n">
+      <c r="AF1" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2" t="s">
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2" t="s">
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2" t="s">
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="2"/>
-      <c r="T3" s="2"/>
-      <c r="U3" s="2" t="s">
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="V3" s="2"/>
-      <c r="W3" s="2"/>
-      <c r="X3" s="2"/>
-      <c r="Y3" s="2"/>
-      <c r="Z3" s="2" t="s">
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+      <c r="Y3" s="3"/>
+      <c r="Z3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="AA3" s="2"/>
-      <c r="AB3" s="2"/>
-      <c r="AC3" s="2"/>
-      <c r="AD3" s="2"/>
-      <c r="AE3" s="2"/>
-      <c r="AF3" s="2"/>
+      <c r="AA3" s="3"/>
+      <c r="AB3" s="3"/>
+      <c r="AC3" s="3"/>
+      <c r="AD3" s="3"/>
+      <c r="AE3" s="3"/>
+      <c r="AF3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="J4" s="0" t="n">
+      <c r="J4" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="O4" s="0" t="n">
+      <c r="O4" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="S4" s="0" t="n">
+      <c r="S4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="W4" s="0" t="n">
+      <c r="W4" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="AC4" s="0" t="n">
+      <c r="AC4" s="1" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2" t="s">
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2" t="s">
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
+      <c r="R8" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="S8" s="2"/>
-      <c r="T8" s="2"/>
-      <c r="U8" s="2" t="s">
+      <c r="S8" s="3"/>
+      <c r="T8" s="3"/>
+      <c r="U8" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="V8" s="2"/>
-      <c r="W8" s="2"/>
-      <c r="X8" s="2"/>
-      <c r="Y8" s="2"/>
-      <c r="Z8" s="2" t="s">
+      <c r="V8" s="3"/>
+      <c r="W8" s="3"/>
+      <c r="X8" s="3"/>
+      <c r="Y8" s="3"/>
+      <c r="Z8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="AA8" s="2"/>
-      <c r="AB8" s="2"/>
-      <c r="AC8" s="2"/>
-      <c r="AD8" s="2"/>
-      <c r="AE8" s="2"/>
-      <c r="AF8" s="2"/>
+      <c r="AA8" s="3"/>
+      <c r="AB8" s="3"/>
+      <c r="AC8" s="3"/>
+      <c r="AD8" s="3"/>
+      <c r="AE8" s="3"/>
+      <c r="AF8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F9" s="0" t="n">
+      <c r="F9" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="O9" s="0" t="n">
+      <c r="O9" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="S9" s="0" t="n">
+      <c r="S9" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="W9" s="0" t="n">
+      <c r="W9" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="AC9" s="0" t="n">
+      <c r="AC9" s="1" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2" t="s">
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2" t="s">
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2" t="s">
+      <c r="N13" s="3"/>
+      <c r="O13" s="3"/>
+      <c r="P13" s="3"/>
+      <c r="Q13" s="3"/>
+      <c r="R13" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="S13" s="2"/>
-      <c r="T13" s="2"/>
-      <c r="U13" s="2" t="s">
+      <c r="S13" s="3"/>
+      <c r="T13" s="3"/>
+      <c r="U13" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="V13" s="2"/>
-      <c r="W13" s="2"/>
-      <c r="X13" s="2"/>
-      <c r="Y13" s="2"/>
-      <c r="Z13" s="2" t="s">
+      <c r="V13" s="3"/>
+      <c r="W13" s="3"/>
+      <c r="X13" s="3"/>
+      <c r="Y13" s="3"/>
+      <c r="Z13" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="AA13" s="2"/>
-      <c r="AB13" s="2"/>
-      <c r="AC13" s="2"/>
-      <c r="AD13" s="2"/>
-      <c r="AE13" s="2"/>
-      <c r="AF13" s="2"/>
+      <c r="AA13" s="3"/>
+      <c r="AB13" s="3"/>
+      <c r="AC13" s="3"/>
+      <c r="AD13" s="3"/>
+      <c r="AE13" s="3"/>
+      <c r="AF13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D14" s="0" t="n">
+      <c r="D14" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="J14" s="0" t="n">
+      <c r="J14" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="O14" s="0" t="n">
+      <c r="O14" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="S14" s="0" t="n">
+      <c r="S14" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="W14" s="0" t="n">
+      <c r="W14" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="AC14" s="0" t="n">
+      <c r="AC14" s="1" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2" t="s">
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2" t="s">
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="M18" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2"/>
-      <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
-      <c r="R18" s="2" t="s">
+      <c r="N18" s="3"/>
+      <c r="O18" s="3"/>
+      <c r="P18" s="3"/>
+      <c r="Q18" s="3"/>
+      <c r="R18" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="S18" s="2"/>
-      <c r="T18" s="2"/>
-      <c r="U18" s="2" t="s">
+      <c r="S18" s="3"/>
+      <c r="T18" s="3"/>
+      <c r="U18" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="V18" s="2"/>
-      <c r="W18" s="2"/>
-      <c r="X18" s="2"/>
-      <c r="Y18" s="4" t="s">
+      <c r="V18" s="3"/>
+      <c r="W18" s="3"/>
+      <c r="X18" s="3"/>
+      <c r="Y18" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="Z18" s="2" t="s">
+      <c r="Z18" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="AA18" s="2"/>
-      <c r="AB18" s="2"/>
-      <c r="AC18" s="2"/>
-      <c r="AD18" s="2"/>
-      <c r="AE18" s="2"/>
-      <c r="AF18" s="2"/>
+      <c r="AA18" s="3"/>
+      <c r="AB18" s="3"/>
+      <c r="AC18" s="3"/>
+      <c r="AD18" s="3"/>
+      <c r="AE18" s="3"/>
+      <c r="AF18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="n">
+      <c r="A19" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B19" s="5" t="n">
+      <c r="B19" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="J19" s="0" t="n">
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="J19" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="O19" s="0" t="n">
+      <c r="O19" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="S19" s="0" t="n">
+      <c r="S19" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="U19" s="5" t="n">
+      <c r="U19" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="V19" s="5"/>
-      <c r="W19" s="5"/>
-      <c r="X19" s="5"/>
-      <c r="Y19" s="0" t="n">
+      <c r="V19" s="6"/>
+      <c r="W19" s="6"/>
+      <c r="X19" s="6"/>
+      <c r="Y19" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AC19" s="0" t="n">
+      <c r="AC19" s="1" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
+    <row r="22" customFormat="false" ht="16.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
-      <c r="N23" s="2"/>
-      <c r="O23" s="2"/>
-      <c r="P23" s="2"/>
-      <c r="Q23" s="2"/>
-      <c r="R23" s="2"/>
-      <c r="S23" s="2"/>
-      <c r="T23" s="2"/>
-      <c r="U23" s="2" t="s">
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="M23" s="3"/>
+      <c r="N23" s="3"/>
+      <c r="O23" s="3"/>
+      <c r="P23" s="3"/>
+      <c r="Q23" s="3"/>
+      <c r="R23" s="3"/>
+      <c r="S23" s="3"/>
+      <c r="T23" s="3"/>
+      <c r="U23" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="V23" s="2"/>
-      <c r="W23" s="2"/>
-      <c r="X23" s="2"/>
-      <c r="Y23" s="2"/>
-      <c r="Z23" s="2" t="s">
+      <c r="V23" s="3"/>
+      <c r="W23" s="3"/>
+      <c r="X23" s="3"/>
+      <c r="Y23" s="3"/>
+      <c r="Z23" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="AA23" s="2"/>
-      <c r="AB23" s="2"/>
-      <c r="AC23" s="2"/>
-      <c r="AD23" s="2"/>
-      <c r="AE23" s="2"/>
-      <c r="AF23" s="2"/>
+      <c r="AA23" s="3"/>
+      <c r="AB23" s="3"/>
+      <c r="AC23" s="3"/>
+      <c r="AD23" s="3"/>
+      <c r="AE23" s="3"/>
+      <c r="AF23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K24" s="0" t="n">
+      <c r="K24" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="W24" s="0" t="n">
+      <c r="W24" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="AC24" s="0" t="n">
+      <c r="AC24" s="1" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
-      <c r="K28" s="2"/>
-      <c r="L28" s="4" t="s">
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="M28" s="2" t="s">
+      <c r="M28" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="N28" s="2"/>
-      <c r="O28" s="2"/>
-      <c r="P28" s="2"/>
-      <c r="Q28" s="2"/>
-      <c r="R28" s="2"/>
-      <c r="S28" s="2"/>
-      <c r="T28" s="2"/>
-      <c r="U28" s="2" t="s">
+      <c r="N28" s="3"/>
+      <c r="O28" s="3"/>
+      <c r="P28" s="3"/>
+      <c r="Q28" s="3"/>
+      <c r="R28" s="3"/>
+      <c r="S28" s="3"/>
+      <c r="T28" s="3"/>
+      <c r="U28" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="V28" s="2"/>
-      <c r="W28" s="2"/>
-      <c r="X28" s="2"/>
-      <c r="Y28" s="2"/>
-      <c r="Z28" s="2" t="s">
+      <c r="V28" s="3"/>
+      <c r="W28" s="3"/>
+      <c r="X28" s="3"/>
+      <c r="Y28" s="3"/>
+      <c r="Z28" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="AA28" s="2"/>
-      <c r="AB28" s="2"/>
-      <c r="AC28" s="2"/>
-      <c r="AD28" s="2"/>
-      <c r="AE28" s="2"/>
-      <c r="AF28" s="2"/>
+      <c r="AA28" s="3"/>
+      <c r="AB28" s="3"/>
+      <c r="AC28" s="3"/>
+      <c r="AD28" s="3"/>
+      <c r="AE28" s="3"/>
+      <c r="AF28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="n">
+      <c r="A29" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G29" s="0" t="n">
+      <c r="G29" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="L29" s="0" t="n">
+      <c r="L29" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="Q29" s="0" t="n">
+      <c r="Q29" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="W29" s="0" t="n">
+      <c r="W29" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="AC29" s="0" t="n">
+      <c r="AC29" s="1" t="n">
         <v>7</v>
       </c>
     </row>
@@ -1611,589 +1639,589 @@
   <dimension ref="A1:C63"/>
   <sheetFormatPr defaultColWidth="9.06640625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="6" width="21.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="6" width="10.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="6" width="22.34"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="6" width="9.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="21.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="10.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="22.34"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="7" width="9.06"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="7" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="7" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="7" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="7" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="7" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="7" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="7" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="7" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="7" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="7" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="7" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="7" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8" t="s">
+      <c r="A23" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="7" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="7" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="7" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="7" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="7" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="7" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="7" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="7" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="s">
+      <c r="A32" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="7" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="6" t="s">
+      <c r="A33" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" s="7" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="6" t="s">
+      <c r="A34" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="C34" s="7" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="6" t="s">
+      <c r="A35" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="C35" s="7" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
+      <c r="A37" s="7" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="s">
+      <c r="A38" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C38" s="6" t="s">
+      <c r="C38" s="7" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="6" t="s">
+      <c r="A39" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C39" s="6" t="s">
+      <c r="C39" s="7" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="6" t="s">
+      <c r="A40" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C40" s="6" t="s">
+      <c r="C40" s="7" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="6" t="s">
+      <c r="A41" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="7" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="6" t="s">
+      <c r="A42" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="C42" s="7" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="6" t="s">
+      <c r="A43" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="B43" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C43" s="6" t="s">
+      <c r="C43" s="7" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="6" t="s">
+      <c r="A44" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="B44" s="6" t="s">
+      <c r="B44" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="7" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="6" t="s">
+      <c r="A45" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="7" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="6" t="s">
+      <c r="A47" s="7" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="6" t="s">
+      <c r="A48" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B48" s="6" t="s">
+      <c r="B48" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C48" s="6" t="s">
+      <c r="C48" s="7" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="6" t="s">
+      <c r="A49" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B49" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C49" s="6" t="s">
+      <c r="C49" s="7" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="6" t="s">
+      <c r="A50" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="B50" s="6" t="s">
+      <c r="B50" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C50" s="6" t="s">
+      <c r="C50" s="7" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="6" t="s">
+      <c r="A51" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="B51" s="6" t="s">
+      <c r="B51" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C51" s="6" t="s">
+      <c r="C51" s="7" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="6" t="s">
+      <c r="A52" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="B52" s="6" t="s">
+      <c r="B52" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C52" s="6" t="s">
+      <c r="C52" s="7" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="6" t="s">
+      <c r="A54" s="7" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="6" t="s">
+      <c r="A55" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B55" s="6" t="s">
+      <c r="B55" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C55" s="6" t="s">
+      <c r="C55" s="7" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="6" t="s">
+      <c r="A56" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="B56" s="6" t="s">
+      <c r="B56" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C56" s="6" t="s">
+      <c r="C56" s="7" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="6" t="s">
+      <c r="A57" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="B57" s="6" t="s">
+      <c r="B57" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C57" s="6" t="s">
+      <c r="C57" s="7" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="6" t="s">
+      <c r="A58" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="B58" s="6" t="s">
+      <c r="B58" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C58" s="6" t="s">
+      <c r="C58" s="7" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="6" t="s">
+      <c r="A59" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="B59" s="6" t="s">
+      <c r="B59" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C59" s="6" t="s">
+      <c r="C59" s="7" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="6" t="s">
+      <c r="A60" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="B60" s="6" t="s">
+      <c r="B60" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C60" s="6" t="s">
+      <c r="C60" s="7" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="6" t="s">
+      <c r="A61" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="B61" s="6" t="s">
+      <c r="B61" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C61" s="6" t="s">
+      <c r="C61" s="7" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="6" t="s">
+      <c r="A63" s="7" t="s">
         <v>127</v>
       </c>
     </row>
@@ -2216,369 +2244,369 @@
   <dimension ref="B1:D33"/>
   <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="36.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="36.63"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="10" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="10" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="10" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="10" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="10" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="10" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="10" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="10" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="10" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="10" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="10" t="s">
         <v>158</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="10" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="10" t="s">
         <v>160</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="10" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="10" t="s">
         <v>163</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="10" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="10" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="10" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="10" t="s">
         <v>172</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="10" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="10" t="s">
         <v>175</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="10" t="s">
         <v>176</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="10" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="10" t="s">
         <v>178</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="10" t="s">
         <v>179</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D18" s="10" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="10" t="s">
         <v>181</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="10" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="10" t="s">
         <v>184</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="10" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="10" t="s">
         <v>187</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D21" s="10" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="D22" s="10" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="10" t="s">
         <v>191</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="10" t="s">
         <v>192</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="D23" s="10" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="10" t="s">
         <v>193</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="C24" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="D24" s="10" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="10" t="s">
         <v>196</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="D25" s="10" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="10" t="s">
         <v>197</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="10" t="s">
         <v>198</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="10" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="10" t="s">
         <v>199</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="D27" s="10" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="9" t="s">
+      <c r="B28" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="C28" s="9" t="s">
+      <c r="C28" s="10" t="s">
         <v>202</v>
       </c>
-      <c r="D28" s="9" t="s">
+      <c r="D28" s="10" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="9" t="s">
+      <c r="B29" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="C29" s="10" t="s">
         <v>204</v>
       </c>
-      <c r="D29" s="9" t="s">
+      <c r="D29" s="10" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="D30" s="9" t="s">
+      <c r="D30" s="10" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="9" t="s">
+      <c r="B31" s="10" t="s">
         <v>207</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="10" t="s">
         <v>208</v>
       </c>
-      <c r="D31" s="9" t="s">
+      <c r="D31" s="10" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="9" t="s">
+      <c r="B32" s="10" t="s">
         <v>209</v>
       </c>
-      <c r="C32" s="9" t="s">
+      <c r="C32" s="10" t="s">
         <v>210</v>
       </c>
-      <c r="D32" s="9" t="s">
+      <c r="D32" s="10" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="9" t="s">
+      <c r="B33" s="10" t="s">
         <v>211</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="C33" s="10" t="s">
         <v>212</v>
       </c>
-      <c r="D33" s="9" t="s">
+      <c r="D33" s="10" t="s">
         <v>151</v>
       </c>
     </row>

</xml_diff>

<commit_message>
support LW, ADDIW, fix bugs
</commit_message>
<xml_diff>
--- a/Tomasulo3CPU/ISA/ISA64.xlsx
+++ b/Tomasulo3CPU/ISA/ISA64.xlsx
@@ -48,7 +48,7 @@
     <t xml:space="preserve">IMM</t>
   </si>
   <si>
-    <t xml:space="preserve">Store: SW</t>
+    <t xml:space="preserve">Store: SW sw rt, offset(rs)</t>
   </si>
   <si>
     <t xml:space="preserve">IMM[11:5]</t>
@@ -72,25 +72,7 @@
     <t xml:space="preserve">IMM[11]</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">U-TYPE: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">LUI / AUIPC</t>
-    </r>
+    <t xml:space="preserve">U-TYPE: LUI / AUIPC</t>
   </si>
   <si>
     <t xml:space="preserve">IMM[31:12]</t>
@@ -713,10 +695,10 @@
       <family val="0"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="10"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="12"/>
@@ -782,7 +764,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -796,6 +778,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1270,15 +1256,15 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
@@ -1347,18 +1333,18 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="6" t="s">
         <v>12</v>
       </c>
       <c r="B18" s="3" t="s">
@@ -1394,7 +1380,7 @@
       <c r="V18" s="3"/>
       <c r="W18" s="3"/>
       <c r="X18" s="3"/>
-      <c r="Y18" s="5" t="s">
+      <c r="Y18" s="6" t="s">
         <v>15</v>
       </c>
       <c r="Z18" s="3" t="s">
@@ -1411,14 +1397,14 @@
       <c r="A19" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B19" s="6" t="n">
+      <c r="B19" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
       <c r="J19" s="1" t="n">
         <v>5</v>
       </c>
@@ -1428,12 +1414,12 @@
       <c r="S19" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="U19" s="6" t="n">
+      <c r="U19" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="V19" s="6"/>
-      <c r="W19" s="6"/>
-      <c r="X19" s="6"/>
+      <c r="V19" s="7"/>
+      <c r="W19" s="7"/>
+      <c r="X19" s="7"/>
       <c r="Y19" s="1" t="n">
         <v>1</v>
       </c>
@@ -1441,16 +1427,16 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
@@ -1504,18 +1490,18 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="s">
+      <c r="A28" s="6" t="s">
         <v>19</v>
       </c>
       <c r="B28" s="3" t="s">
@@ -1530,7 +1516,7 @@
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
       <c r="K28" s="3"/>
-      <c r="L28" s="5" t="s">
+      <c r="L28" s="6" t="s">
         <v>15</v>
       </c>
       <c r="M28" s="3" t="s">
@@ -1639,589 +1625,589 @@
   <dimension ref="A1:C63"/>
   <sheetFormatPr defaultColWidth="9.06640625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="21.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="10.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="22.34"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="7" width="9.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="21.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="8" width="10.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="8" width="22.34"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="8" width="9.06"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="8" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="8" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="8" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="8" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="8" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="8" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="8" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="8" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="8" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="8" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="8" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="8" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="8" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="8" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="8" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="8" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="8" t="s">
+      <c r="A22" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="8" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9" t="s">
+      <c r="A23" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="8" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="8" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="8" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" s="8" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="8" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="s">
+      <c r="A29" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="C29" s="8" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="s">
+      <c r="A30" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" s="8" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7" t="s">
+      <c r="A31" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="B31" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="C31" s="8" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="s">
+      <c r="A32" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B32" s="7" t="s">
+      <c r="B32" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="C32" s="8" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="s">
+      <c r="A33" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C33" s="7" t="s">
+      <c r="C33" s="8" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7" t="s">
+      <c r="A34" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C34" s="8" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7" t="s">
+      <c r="A35" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B35" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="C35" s="8" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7" t="s">
+      <c r="A37" s="8" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="7" t="s">
+      <c r="A38" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="B38" s="7" t="s">
+      <c r="B38" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="C38" s="8" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="7" t="s">
+      <c r="A39" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B39" s="7" t="s">
+      <c r="B39" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C39" s="7" t="s">
+      <c r="C39" s="8" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="7" t="s">
+      <c r="A40" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="B40" s="7" t="s">
+      <c r="B40" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C40" s="7" t="s">
+      <c r="C40" s="8" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="7" t="s">
+      <c r="A41" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="7" t="s">
+      <c r="B41" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C41" s="7" t="s">
+      <c r="C41" s="8" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="7" t="s">
+      <c r="A42" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="B42" s="7" t="s">
+      <c r="B42" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C42" s="7" t="s">
+      <c r="C42" s="8" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="7" t="s">
+      <c r="A43" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B43" s="7" t="s">
+      <c r="B43" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="C43" s="7" t="s">
+      <c r="C43" s="8" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7" t="s">
+      <c r="A44" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="B44" s="7" t="s">
+      <c r="B44" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C44" s="7" t="s">
+      <c r="C44" s="8" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="7" t="s">
+      <c r="A45" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="B45" s="7" t="s">
+      <c r="B45" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="C45" s="7" t="s">
+      <c r="C45" s="8" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7" t="s">
+      <c r="A47" s="8" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="7" t="s">
+      <c r="A48" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="B48" s="7" t="s">
+      <c r="B48" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C48" s="7" t="s">
+      <c r="C48" s="8" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="7" t="s">
+      <c r="A49" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="B49" s="7" t="s">
+      <c r="B49" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C49" s="7" t="s">
+      <c r="C49" s="8" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="7" t="s">
+      <c r="A50" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="B50" s="7" t="s">
+      <c r="B50" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C50" s="7" t="s">
+      <c r="C50" s="8" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="7" t="s">
+      <c r="A51" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="B51" s="7" t="s">
+      <c r="B51" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C51" s="7" t="s">
+      <c r="C51" s="8" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="7" t="s">
+      <c r="A52" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="B52" s="7" t="s">
+      <c r="B52" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C52" s="7" t="s">
+      <c r="C52" s="8" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="7" t="s">
+      <c r="A54" s="8" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="7" t="s">
+      <c r="A55" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="B55" s="7" t="s">
+      <c r="B55" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C55" s="7" t="s">
+      <c r="C55" s="8" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="7" t="s">
+      <c r="A56" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="B56" s="7" t="s">
+      <c r="B56" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C56" s="7" t="s">
+      <c r="C56" s="8" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="7" t="s">
+      <c r="A57" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="B57" s="7" t="s">
+      <c r="B57" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C57" s="7" t="s">
+      <c r="C57" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="7" t="s">
+      <c r="A58" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="B58" s="7" t="s">
+      <c r="B58" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="C58" s="7" t="s">
+      <c r="C58" s="8" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="7" t="s">
+      <c r="A59" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="B59" s="7" t="s">
+      <c r="B59" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C59" s="7" t="s">
+      <c r="C59" s="8" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="7" t="s">
+      <c r="A60" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="B60" s="7" t="s">
+      <c r="B60" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="C60" s="7" t="s">
+      <c r="C60" s="8" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="7" t="s">
+      <c r="A61" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="B61" s="7" t="s">
+      <c r="B61" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="C61" s="7" t="s">
+      <c r="C61" s="8" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="7" t="s">
+      <c r="A63" s="8" t="s">
         <v>127</v>
       </c>
     </row>
@@ -2248,365 +2234,365 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="11" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="11" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="11" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="11" t="s">
         <v>140</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="11" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="11" t="s">
         <v>144</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="11" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="11" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="11" t="s">
         <v>150</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="11" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="11" t="s">
         <v>152</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="11" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="11" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="11" t="s">
         <v>158</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="11" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="11" t="s">
         <v>161</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="11" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="11" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="11" t="s">
         <v>167</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="11" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="11" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="11" t="s">
         <v>172</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="11" t="s">
         <v>173</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="11" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="11" t="s">
         <v>175</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="11" t="s">
         <v>176</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="11" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="11" t="s">
         <v>178</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="11" t="s">
         <v>179</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="11" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="11" t="s">
         <v>181</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="11" t="s">
         <v>182</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="11" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="11" t="s">
         <v>184</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="11" t="s">
         <v>185</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="11" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="11" t="s">
         <v>187</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="11" t="s">
         <v>188</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="11" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="11" t="s">
         <v>189</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="11" t="s">
         <v>190</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="11" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="11" t="s">
         <v>192</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="11" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="11" t="s">
         <v>193</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" s="11" t="s">
         <v>194</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="11" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="11" t="s">
         <v>196</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="11" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="11" t="s">
         <v>198</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="11" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="11" t="s">
         <v>199</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" s="11" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="11" t="s">
         <v>201</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="11" t="s">
         <v>202</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D28" s="11" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="11" t="s">
         <v>203</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="11" t="s">
         <v>204</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D29" s="11" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="11" t="s">
         <v>205</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="11" t="s">
         <v>206</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="D30" s="11" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="11" t="s">
         <v>207</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="D31" s="10" t="s">
+      <c r="D31" s="11" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="10" t="s">
+      <c r="B32" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="C32" s="11" t="s">
         <v>210</v>
       </c>
-      <c r="D32" s="10" t="s">
+      <c r="D32" s="11" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="10" t="s">
+      <c r="B33" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C33" s="11" t="s">
         <v>212</v>
       </c>
-      <c r="D33" s="10" t="s">
+      <c r="D33" s="11" t="s">
         <v>151</v>
       </c>
     </row>

</xml_diff>

<commit_message>
passed a bubble sort cprogram
</commit_message>
<xml_diff>
--- a/Tomasulo3CPU/ISA/ISA64.xlsx
+++ b/Tomasulo3CPU/ISA/ISA64.xlsx
@@ -5,12 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="RISCV64" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Opcode" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Arch_REG" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Sheet5" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Sheet4" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="257">
   <si>
     <t xml:space="preserve">R-TYPE: ADD, SUB, AND ,OR, SLT, MUL, DI</t>
   </si>
@@ -661,6 +663,138 @@
   </si>
   <si>
     <t xml:space="preserve">t6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">976(122)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40000113           addi sp,zero,1024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00400793           addi a5,zero,4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fee6d8e3           bge a3,a4,20 &lt;bubble_sort+0x18&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0600006f           jal zero,64 &lt;main&gt; </t>
+  </si>
+  <si>
+    <t xml:space="preserve">00f12e23           sw a5,28(sp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00d7a023           sw a3,0(a5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fd010113           addi sp,sp,-48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00700793           addi a5,zero,7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00e7a223           sw a4,4(a5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">02113423           sd ra,40(sp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00f12023           sw a5,0(sp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fe5ff06f           jal zero,20 &lt;bubble_sort+0x18&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00300793           addi a5,zero,3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00010513           addi a0,sp,0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fff5859b           addiw a1,a1,-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00f12223           sw a5,4(sp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f59ff0ef           jal ra,8 &lt;bubble_sort&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ffc60613           addi a2,a2,-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00500793           addi a5,zero,5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fff5879b           addiw a5,a1,-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00058c63           beq a1,zero,60 &lt;bubble_sort+0x58&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00f12423           sw a5,8(sp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04f05a63           bge zero,a5,60 &lt;bubble_sort+0x58&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00050793           addi a5,a0,0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00100793           addi a5,zero,1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00078593           addi a1,a5,0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fcb04ce3           blt zero,a1,28 &lt;bubble_sort+0x20&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00f12623           sw a5,12(sp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00279793           slli a5,a5,0x2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00800593           addi a1,zero,8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00f50633           add a2,a0,a5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00b12823           sw a1,16(sp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0300006f           jal zero,4c &lt;bubble_sort+0x44&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ff1ff06f           jal zero,4c &lt;bubble_sort+0x44&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00200793           addi a5,zero,2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00478793           addi a5,a5,4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00008067           jalr zero,0(ra)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00f12a23           sw a5,20(sp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00c78e63           beq a5,a2,40 &lt;bubble_sort+0x38&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00600793           addi a5,zero,6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0007a703           lw a4,0(a5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00f12c23           sw a5,24(sp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0047a683           lw a3,4(a5)</t>
   </si>
 </sst>
 </file>
@@ -671,7 +805,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -699,6 +833,7 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="12"/>
@@ -706,6 +841,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -764,7 +905,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -810,6 +951,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1427,7 +1576,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
         <v>16</v>
       </c>
@@ -2605,4 +2754,327 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="B1" s="0" t="n">
+        <f aca="false">1024-48</f>
+        <v>976</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>167</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <f aca="false">976+28</f>
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>213</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="62.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="46.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="45.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46.57"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>215</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>217</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>220</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>221</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>223</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>224</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>227</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>229</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>232</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>233</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>235</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>238</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>239</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>241</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>242</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>243</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>244</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>246</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>248</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>249</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>251</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>253</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>255</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>256</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>